<commit_message>
Refit the EM2040 on 16 sessions, and two guards that made it trustworthy
Cruise pool 4.85 h -> 131.9 h, spanning 1279-3080 rpm against 1400-2500.
Efficiency moves up to 11.8% at 5 and 10 kt - the ends correcting where the old
law extrapolated, not the middle moving. Adopted on evidence: against the
measured bin medians, speed RMS 0.363 -> 0.290 kt and fuel 0.142 -> 0.115 L/h.

Two data faults are now rejected by a guard rather than by hand: 08-14 reported
12-14 L/h at 1889 rpm and 4.1 kt, and 08-15 reported 0.00 L/h while cruising.

The gauge deliberately did NOT change. The record now contains refuels, so
litres-per-point is only defined within a falling stretch; tools/drawdown.py
owns that segmentation and every consumer reads it. Properly cut it gives
2.34 +/- 0.16 L/point over 37-100%, which is 1.7 sigma from the 2.06 in force
and reads 1.85 inside the old band - not enough to move a number that would
plan every mission longer.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DriX8_Endurance_EM2040.xlsx
+++ b/docs/DriX8_Endurance_EM2040.xlsx
@@ -676,10 +676,10 @@
         <v>4</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1079</v>
+        <v>1084</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>1.067051154</v>
+        <v>1.225442136</v>
       </c>
       <c r="K4" s="3">
         <f>H4/J4</f>
@@ -696,14 +696,14 @@
         <v>1000</v>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1.907687088</v>
+        <v>1.898517679</v>
       </c>
       <c r="C5" s="3">
         <f>B5*$B$15</f>
         <v/>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0.971029406</v>
+        <v>1.125200708</v>
       </c>
       <c r="E5" s="3">
         <f>D5*100/$B$16</f>
@@ -722,10 +722,10 @@
         <v>5</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>1348</v>
+        <v>1355</v>
       </c>
       <c r="J5" s="3" t="n">
-        <v>1.448888037</v>
+        <v>1.591372501</v>
       </c>
       <c r="K5" s="3">
         <f>H5/J5</f>
@@ -742,14 +742,14 @@
         <v>1250</v>
       </c>
       <c r="B6" s="3" t="n">
-        <v>2.38460886</v>
+        <v>2.373147099</v>
       </c>
       <c r="C6" s="3">
         <f>B6*$B$15</f>
         <v/>
       </c>
       <c r="D6" s="3" t="n">
-        <v>1.299149316</v>
+        <v>1.440935247</v>
       </c>
       <c r="E6" s="3">
         <f>D6*100/$B$16</f>
@@ -768,10 +768,10 @@
         <v>6</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>1618</v>
+        <v>1626</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>1.934341305</v>
+        <v>2.046996169</v>
       </c>
       <c r="K6" s="3">
         <f>H6/J6</f>
@@ -783,14 +783,14 @@
         <v>1500</v>
       </c>
       <c r="B7" s="3" t="n">
-        <v>2.861530631</v>
+        <v>2.847776519</v>
       </c>
       <c r="C7" s="3">
         <f>B7*$B$15</f>
         <v/>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1.707296906</v>
+        <v>1.822169146</v>
       </c>
       <c r="E7" s="3">
         <f>D7*100/$B$16</f>
@@ -804,10 +804,10 @@
         <v>7</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>1888</v>
+        <v>1897</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>2.552204331</v>
+        <v>2.625245824</v>
       </c>
       <c r="K7" s="3">
         <f>H7/J7</f>
@@ -819,14 +819,14 @@
         <v>1750</v>
       </c>
       <c r="B8" s="3" t="n">
-        <v>3.338452403</v>
+        <v>3.322405939</v>
       </c>
       <c r="C8" s="3">
         <f>B8*$B$15</f>
         <v/>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2.218413502</v>
+        <v>2.294765211</v>
       </c>
       <c r="E8" s="3">
         <f>D8*100/$B$16</f>
@@ -840,10 +840,10 @@
         <v>8</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>2157</v>
+        <v>2168</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>3.33127049</v>
+        <v>3.359054152</v>
       </c>
       <c r="K8" s="3">
         <f>H8/J8</f>
@@ -855,14 +855,14 @@
         <v>2000</v>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3.815374175</v>
+        <v>3.797035359</v>
       </c>
       <c r="C9" s="3">
         <f>B9*$B$15</f>
         <v/>
       </c>
       <c r="D9" s="3" t="n">
-        <v>2.855440434</v>
+        <v>2.88458625</v>
       </c>
       <c r="E9" s="3">
         <f>D9*100/$B$16</f>
@@ -876,10 +876,10 @@
         <v>9</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>2427</v>
+        <v>2439</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>4.300333155</v>
+        <v>4.281353838</v>
       </c>
       <c r="K9" s="3">
         <f>H9/J9</f>
@@ -891,14 +891,14 @@
         <v>2250</v>
       </c>
       <c r="B10" s="3" t="n">
-        <v>4.292295947</v>
+        <v>4.271664778</v>
       </c>
       <c r="C10" s="3">
         <f>B10*$B$15</f>
         <v/>
       </c>
       <c r="D10" s="3" t="n">
-        <v>3.64131903</v>
+        <v>3.61749507</v>
       </c>
       <c r="E10" s="3">
         <f>D10*100/$B$16</f>
@@ -912,10 +912,10 @@
         <v>10</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>2697</v>
+        <v>2710</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>5.488185698</v>
+        <v>5.425077567</v>
       </c>
       <c r="K10" s="3">
         <f>H10/J10</f>
@@ -927,14 +927,14 @@
         <v>2500</v>
       </c>
       <c r="B11" s="3" t="n">
-        <v>4.769217719</v>
+        <v>4.746294198</v>
       </c>
       <c r="C11" s="3">
         <f>B11*$B$15</f>
         <v/>
       </c>
       <c r="D11" s="3" t="n">
-        <v>4.598990616</v>
+        <v>4.519354477</v>
       </c>
       <c r="E11" s="3">
         <f>D11*100/$B$16</f>
@@ -948,10 +948,10 @@
         <v>11</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>2966</v>
+        <v>2981</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>6.923621495</v>
+        <v>6.823158025</v>
       </c>
       <c r="K11" s="3">
         <f>H11/J11</f>
@@ -963,14 +963,14 @@
         <v>2750</v>
       </c>
       <c r="B12" s="3" t="n">
-        <v>5.246139491</v>
+        <v>5.220923618</v>
       </c>
       <c r="C12" s="3">
         <f>B12*$B$15</f>
         <v/>
       </c>
       <c r="D12" s="3" t="n">
-        <v>5.751396522</v>
+        <v>5.616027278</v>
       </c>
       <c r="E12" s="3">
         <f>D12*100/$B$16</f>
@@ -991,14 +991,14 @@
         <v>3000</v>
       </c>
       <c r="B13" s="3" t="n">
-        <v>5.723061263</v>
+        <v>5.695553038</v>
       </c>
       <c r="C13" s="3">
         <f>B13*$B$15</f>
         <v/>
       </c>
       <c r="D13" s="3" t="n">
-        <v>7.121478076</v>
+        <v>6.933376282</v>
       </c>
       <c r="E13" s="3">
         <f>D13*100/$B$16</f>
@@ -1039,35 +1039,35 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Source: DriX-8 MCAP logs 04-09 Aug 2026 (EM2040 fitted) — 4.85 h steady cruise, flow meter vs thruster RPM.</t>
+          <t>Source: DriX-8 MCAP logs (EM2040 fitted) — 131.90 h steady cruise over 1279-3080 rpm, flow meter vs thruster RPM.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Fuel law (through origin) L/H = 1.0038e-03·RPM -2.7743e-07·RPM² +2.4471e-10·RPM³  (R² 0.9996),</t>
+          <t>Fuel law (through origin) L/H = 1.3598e-03·RPM -5.1052e-07·RPM² +2.7587e-10·RPM³,</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>anchored by (0,0) and the measured 0.95 L/H station-keeping figure at ~1005 rpm.</t>
+          <t>anchored by (0,0) and the measured 1.05 L/H station-keeping figure at ~1010 rpm.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Speed law (through origin) KNOTS = 0.003708·RPM  (R² 0.949; SOG-based, ±5-8% tidal).</t>
+          <t>Speed law (through origin) KNOTS = 0.003690·RPM  (SOG-based, ±5-8% tidal).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Both agree with the primary in-band laws (planner model.json) to ≤3.7% in-window, 0.3% at 8 kt.</t>
+          <t>Against the planner's own laws (model.json): 0.5% at 8 kt, ≤1.1% above 1600 rpm, worst 10.8% at 1280 rpm where the through-origin constraint bends toward idle.</t>
         </is>
       </c>
     </row>

</xml_diff>